<commit_message>
correcion de archivos v4
</commit_message>
<xml_diff>
--- a/Documentos/ProductBacklogCorregido.xlsx
+++ b/Documentos/ProductBacklogCorregido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveespochedu-my.sharepoint.com/personal/jonathan_aucancela_espoch_edu_ec/Documents/Documentos/Espoch/Octavo/Aplicaciones informáticas 2/Parcial 1/Tareas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{3B73CD9B-AD82-416D-96B8-D24AE7031C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B2ED496-8015-4EDC-AEEC-DC58FE0D766E}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="8_{3B73CD9B-AD82-416D-96B8-D24AE7031C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB6FAC07-CC05-4FB7-8775-EA4003927049}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{7A8F741B-9112-4896-B995-875A9BDE94F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="75">
   <si>
     <t>Product Backlog - SecuraBank</t>
   </si>
@@ -62,21 +62,12 @@
     <t>2 Gestión de autenticación y acceso</t>
   </si>
   <si>
-    <t>Implementar Control de Acceso Basado en Roles (RBAC)</t>
-  </si>
-  <si>
-    <t>Validar la autenticación con MFA para el acceso de usuarios.</t>
-  </si>
-  <si>
     <t>Establecer reglas de bloqueo por intentos fallidos de inicio de sesión.</t>
   </si>
   <si>
     <t>3 Seguridad en datos y transacciones</t>
   </si>
   <si>
-    <t>Implementar cifrado de datos sensibles usando AES-256.</t>
-  </si>
-  <si>
     <t>Proteger el sistema contra inyección SQL y ataques XSS.</t>
   </si>
   <si>
@@ -215,12 +206,6 @@
     <t>22 de octubre 2024</t>
   </si>
   <si>
-    <t>5 de diciembre 2024</t>
-  </si>
-  <si>
-    <t>26 de diciembre 2024</t>
-  </si>
-  <si>
     <t>HT5</t>
   </si>
   <si>
@@ -236,9 +221,6 @@
     <t>HT7</t>
   </si>
   <si>
-    <t>Crear del prototipo  inicial dl sistema y la base de datos para usuarios y transacciones.</t>
-  </si>
-  <si>
     <t>Configurar el entorno de desarrollo y herramientas necesarias</t>
   </si>
   <si>
@@ -254,7 +236,31 @@
     <t>Diseñar la base de datos inicial y el repositorio del proyecto</t>
   </si>
   <si>
-    <t>12 de diciembre 2024</t>
+    <t>5 de noviembre 2024</t>
+  </si>
+  <si>
+    <t>12 de noviembre 2024</t>
+  </si>
+  <si>
+    <t>26 de noviembre 2024</t>
+  </si>
+  <si>
+    <t>27 de noviembre de2024</t>
+  </si>
+  <si>
+    <t>28 de noviembre de2024</t>
+  </si>
+  <si>
+    <t>30 de noviembre de 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crear del prototipo  inicial de la base de datos </t>
+  </si>
+  <si>
+    <t>Creacion del esquema según el patrón de diseño.</t>
+  </si>
+  <si>
+    <t>Crear el entorno de desarrollo  Django para el frontend</t>
   </si>
 </sst>
 </file>
@@ -451,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -477,6 +483,24 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -486,23 +510,8 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -842,13 +851,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83A87B21-3BDC-40F9-B20F-2399C52423D9}">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.77734375" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
     <col min="5" max="5" width="13.109375" customWidth="1"/>
-    <col min="7" max="7" width="20.21875" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -873,203 +882,217 @@
         <v>3</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>6</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="E3" s="2">
+        <v>4</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="16"/>
+      <c r="B4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="2">
+        <v>4</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="16"/>
+      <c r="B5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="16"/>
+      <c r="B6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="2">
+        <v>4</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17"/>
+      <c r="B7" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="C7" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="2">
+        <v>4</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="2">
-        <v>4</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="C8" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="2">
+        <v>4</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11"/>
+      <c r="B9" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10"/>
-      <c r="B4" s="2" t="s">
+      <c r="C9" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E4" s="2">
-        <v>4</v>
-      </c>
-      <c r="F4" s="2">
-        <v>1</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="2">
-        <v>4</v>
-      </c>
-      <c r="F5" s="2">
-        <v>1</v>
-      </c>
-      <c r="G5" s="2" t="s">
+      <c r="D9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2">
+        <v>4</v>
+      </c>
+      <c r="F9" s="2">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="11"/>
+      <c r="B10" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10"/>
-      <c r="B6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="C10" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E10" s="2">
+        <v>4</v>
+      </c>
+      <c r="F10" s="2">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="2">
-        <v>4</v>
-      </c>
-      <c r="F6" s="2">
-        <v>1</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11"/>
-      <c r="B7" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" s="2">
-        <v>4</v>
-      </c>
-      <c r="F7" s="2">
-        <v>1</v>
-      </c>
-      <c r="G7" s="2" t="s">
+    </row>
+    <row r="11" spans="1:7" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12"/>
+      <c r="B11" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="2">
-        <v>20</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="2">
-        <v>4</v>
-      </c>
-      <c r="F9" s="2">
-        <v>1</v>
-      </c>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
-      <c r="B10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="2">
-        <v>4</v>
-      </c>
-      <c r="F10" s="2">
+      <c r="C11" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="2">
+        <v>4</v>
+      </c>
+      <c r="F11" s="2">
         <v>2</v>
       </c>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="14"/>
-      <c r="B11" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="G11" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="2">
-        <v>4</v>
-      </c>
-      <c r="F11" s="2">
-        <v>1</v>
-      </c>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="15"/>
-      <c r="B12" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="17" t="s">
+      <c r="B12" s="2"/>
+      <c r="C12" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -1079,33 +1102,33 @@
         <v>4</v>
       </c>
       <c r="F12" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="9"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="E13" s="2">
         <v>4</v>
       </c>
       <c r="F13" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="12"/>
+      <c r="A14" s="9" t="s">
+        <v>16</v>
+      </c>
       <c r="B14" s="2"/>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1120,9 +1143,9 @@
       <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="12"/>
+      <c r="A15" s="9"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -1137,68 +1160,66 @@
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="9"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="2">
+        <v>4</v>
+      </c>
+      <c r="F16" s="2">
+        <v>1</v>
+      </c>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" s="2">
+        <v>4</v>
+      </c>
+      <c r="F17" s="2">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="9"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16" s="2">
-        <v>4</v>
-      </c>
-      <c r="F16" s="2">
-        <v>1</v>
-      </c>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="12"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17" s="2">
-        <v>4</v>
-      </c>
-      <c r="F17" s="2">
-        <v>1</v>
-      </c>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="12"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="E18" s="2">
         <v>4</v>
       </c>
       <c r="F18" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
+    <row r="19" spans="1:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="E19" s="2">
         <v>4</v>
@@ -1208,31 +1229,33 @@
       </c>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="12"/>
+    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="B20" s="2"/>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" s="2">
+        <v>4</v>
+      </c>
+      <c r="F20" s="2">
+        <v>1</v>
+      </c>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="9"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="E20" s="2">
-        <v>4</v>
-      </c>
-      <c r="F20" s="2">
-        <v>2</v>
-      </c>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="12"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="E21" s="2">
         <v>4</v>
@@ -1242,158 +1265,156 @@
       </c>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="12" t="s">
+    <row r="22" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="9"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="2">
+        <v>4</v>
+      </c>
+      <c r="F22" s="2">
+        <v>2</v>
+      </c>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="2">
+        <v>4</v>
+      </c>
+      <c r="F23" s="2">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="9"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="2">
+        <v>4</v>
+      </c>
+      <c r="F24" s="2">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2"/>
+    </row>
+    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="9"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="2">
+        <v>4</v>
+      </c>
+      <c r="F25" s="2">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2"/>
+    </row>
+    <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="2">
+        <v>4</v>
+      </c>
+      <c r="F26" s="2">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2"/>
+    </row>
+    <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="9"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="2">
+        <v>4</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2"/>
+    </row>
+    <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E22" s="2">
-        <v>4</v>
-      </c>
-      <c r="F22" s="2">
-        <v>1</v>
-      </c>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="12"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="2">
-        <v>4</v>
-      </c>
-      <c r="F23" s="2">
+      <c r="B28" s="2"/>
+      <c r="C28" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28" s="2">
+        <v>4</v>
+      </c>
+      <c r="F28" s="2">
         <v>2</v>
       </c>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="12"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" s="2">
-        <v>4</v>
-      </c>
-      <c r="F24" s="2">
-        <v>2</v>
-      </c>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E25" s="2">
-        <v>4</v>
-      </c>
-      <c r="F25" s="2">
-        <v>1</v>
-      </c>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="12"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E26" s="2">
-        <v>4</v>
-      </c>
-      <c r="F26" s="2">
-        <v>1</v>
-      </c>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="12"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" s="2">
-        <v>4</v>
-      </c>
-      <c r="F27" s="2">
-        <v>1</v>
-      </c>
-      <c r="G27" s="2"/>
-    </row>
-    <row r="28" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="1" t="s">
+      <c r="G28" s="2"/>
+    </row>
+    <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="9"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E28" s="2">
-        <v>4</v>
-      </c>
-      <c r="F28" s="2">
-        <v>1</v>
-      </c>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="12"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="2">
+        <v>4</v>
+      </c>
+      <c r="F29" s="2">
+        <v>1</v>
+      </c>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="9"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="E29" s="2">
-        <v>4</v>
-      </c>
-      <c r="F29" s="2">
-        <v>1</v>
-      </c>
-      <c r="G29" s="2"/>
-    </row>
-    <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="E30" s="2">
         <v>4</v>
@@ -1403,50 +1424,52 @@
       </c>
       <c r="G30" s="2"/>
     </row>
-    <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="12"/>
+    <row r="31" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>44</v>
+      </c>
       <c r="B31" s="2"/>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E31" s="2">
+        <v>4</v>
+      </c>
+      <c r="F31" s="2">
+        <v>2</v>
+      </c>
+      <c r="G31" s="2"/>
+    </row>
+    <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="9"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="2">
-        <v>4</v>
-      </c>
-      <c r="F31" s="2">
-        <v>1</v>
-      </c>
-      <c r="G31" s="2"/>
-    </row>
-    <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="12"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" s="2">
+        <v>4</v>
+      </c>
+      <c r="F32" s="2">
+        <v>1</v>
+      </c>
+      <c r="G32" s="2"/>
+    </row>
+    <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="E32" s="2">
-        <v>4</v>
-      </c>
-      <c r="F32" s="2">
-        <v>2</v>
-      </c>
-      <c r="G32" s="2"/>
-    </row>
-    <row r="33" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="E33" s="2">
         <v>4</v>
@@ -1457,32 +1480,30 @@
       <c r="G33" s="2"/>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="12"/>
+      <c r="A34" s="9"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E34" s="2">
+        <v>4</v>
+      </c>
+      <c r="F34" s="2">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="9"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="E34" s="2">
-        <v>4</v>
-      </c>
-      <c r="F34" s="2">
-        <v>1</v>
-      </c>
-      <c r="G34" s="2"/>
-    </row>
-    <row r="35" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B35" s="2"/>
-      <c r="C35" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="E35" s="2">
         <v>4</v>
@@ -1492,51 +1513,51 @@
       </c>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="12"/>
+    <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="B36" s="2"/>
-      <c r="C36" s="17" t="s">
+      <c r="C36" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D36" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E36" s="2">
+        <v>4</v>
+      </c>
+      <c r="F36" s="2">
+        <v>1</v>
+      </c>
+      <c r="G36" s="2"/>
+    </row>
+    <row r="37" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="9"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E36" s="2">
-        <v>4</v>
-      </c>
-      <c r="F36" s="2">
-        <v>1</v>
-      </c>
-      <c r="G36" s="2"/>
-    </row>
-    <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A37" s="12"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" s="2">
+        <v>4</v>
+      </c>
+      <c r="F37" s="2">
+        <v>1</v>
+      </c>
+      <c r="G37" s="2"/>
+    </row>
+    <row r="38" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="9"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E37" s="2">
-        <v>4</v>
-      </c>
-      <c r="F37" s="2">
-        <v>2</v>
-      </c>
-      <c r="G37" s="2"/>
-    </row>
-    <row r="38" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B38" s="2"/>
-      <c r="C38" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="E38" s="2">
         <v>4</v>
       </c>
@@ -1544,40 +1565,6 @@
         <v>1</v>
       </c>
       <c r="G38" s="2"/>
-    </row>
-    <row r="39" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="12"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E39" s="2">
-        <v>4</v>
-      </c>
-      <c r="F39" s="2">
-        <v>1</v>
-      </c>
-      <c r="G39" s="2"/>
-    </row>
-    <row r="40" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A40" s="12"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E40" s="2">
-        <v>4</v>
-      </c>
-      <c r="F40" s="2">
-        <v>1</v>
-      </c>
-      <c r="G40" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>